<commit_message>
Add Gemini service and enhance AI analysis features
Introduces Google Gemini AI integration via gemini_service.py and updates environment/configuration for Gemini and Azure OpenAI. Improves prompt structure and parsing logic in azure_openai_service.py for more actionable, location-specific business advice. Refactors work_suggestion_detail.html for richer UI presentation of AI analysis. Updates database and API version settings, adds new management command, and provides test scaffolding for Gemini features.
</commit_message>
<xml_diff>
--- a/core/home/ex/aka.xlsx
+++ b/core/home/ex/aka.xlsx
@@ -1116,8 +1116,8 @@
   <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.85546875" customWidth="1"/>
-    <col min="2" max="2" width="38.140625" customWidth="1"/>
+    <col min="1" max="1" width="44.28515625" customWidth="1"/>
+    <col min="2" max="2" width="53.28515625" customWidth="1"/>
     <col min="3" max="3" width="31" customWidth="1"/>
     <col min="6" max="6" width="33.7109375" customWidth="1"/>
     <col min="7" max="7" width="25.5703125" customWidth="1"/>
@@ -1297,7 +1297,7 @@
         <v>60</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1308,7 +1308,7 @@
         <v>61</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1341,7 +1341,7 @@
         <v>64</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1352,7 +1352,7 @@
         <v>65</v>
       </c>
       <c r="C20">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1363,7 +1363,7 @@
         <v>66</v>
       </c>
       <c r="C21">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1374,7 +1374,7 @@
         <v>67</v>
       </c>
       <c r="C22">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1385,7 +1385,7 @@
         <v>68</v>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1396,7 +1396,7 @@
         <v>69</v>
       </c>
       <c r="C24">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1407,7 +1407,7 @@
         <v>70</v>
       </c>
       <c r="C25">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1418,7 +1418,7 @@
         <v>71</v>
       </c>
       <c r="C26">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1429,7 +1429,7 @@
         <v>72</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1462,7 +1462,7 @@
         <v>75</v>
       </c>
       <c r="C30">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1473,7 +1473,7 @@
         <v>76</v>
       </c>
       <c r="C31">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1484,7 +1484,7 @@
         <v>77</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1495,7 +1495,7 @@
         <v>78</v>
       </c>
       <c r="C33">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1506,7 +1506,7 @@
         <v>79</v>
       </c>
       <c r="C34">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1528,7 +1528,7 @@
         <v>81</v>
       </c>
       <c r="C36">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1539,7 +1539,7 @@
         <v>72</v>
       </c>
       <c r="C37">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1550,7 +1550,7 @@
         <v>82</v>
       </c>
       <c r="C38">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1561,7 +1561,7 @@
         <v>83</v>
       </c>
       <c r="C39">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1572,7 +1572,7 @@
         <v>84</v>
       </c>
       <c r="C40">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1583,7 +1583,7 @@
         <v>85</v>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1594,7 +1594,7 @@
         <v>86</v>
       </c>
       <c r="C42">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1605,7 +1605,7 @@
         <v>87</v>
       </c>
       <c r="C43">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1616,7 +1616,7 @@
         <v>88</v>
       </c>
       <c r="C44">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>